<commit_message>
Playtesting -ruin update 26-02-26b
- Always show Sealed Gate quickexit (it's in the logic).
</commit_message>
<xml_diff>
--- a/claude_reference/Ruin_playtesting_checklist.xlsx
+++ b/claude_reference/Ruin_playtesting_checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hansr\Documents\GitHub\WorldsCollide\claude_reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5314EE24-5E78-4511-88DD-AEC50203A95F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33FE585B-B5DA-44A5-8200-5E7F8787636F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{690EC4E7-DE9A-4E52-B9DA-56D934A5EC63}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{690EC4E7-DE9A-4E52-B9DA-56D934A5EC63}"/>
   </bookViews>
   <sheets>
     <sheet name="Rewards" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="166">
   <si>
     <t>PLAYTESTING CHECKLIST: Rewards in -ruin mode</t>
   </si>
@@ -526,6 +526,15 @@
   </si>
   <si>
     <t>ms-wor-52': {"Mobliz WOR": [RewardType.CHARACTER, RewardType.ESPER, RewardType.ITEM]},   # Mobliz WoR.  Actually '237R' if interiors randomized.</t>
+  </si>
+  <si>
+    <t>Always show Sealed Gate trap exit</t>
+  </si>
+  <si>
+    <t>edit in sealed_gate.ruination_mod</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Party formation after Phunbaba is broken!  </t>
   </si>
 </sst>
 </file>
@@ -941,7 +950,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F93C4B77-39C0-44C7-B9BF-61991AECD056}">
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13" style="1" customWidth="1"/>
@@ -950,12 +959,12 @@
     <col min="5" max="5" width="11.54296875" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>46</v>
       </c>
@@ -972,10 +981,13 @@
         <v>51</v>
       </c>
       <c r="F3" t="s">
+        <v>146</v>
+      </c>
+      <c r="J3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>56</v>
       </c>
@@ -991,11 +1003,11 @@
       <c r="E4" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="F4" t="s">
+      <c r="J4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>56</v>
       </c>
@@ -1008,12 +1020,15 @@
       <c r="E5" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="F5" t="s">
+      <c r="J5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>56</v>
       </c>
       <c r="C6" t="s">
@@ -1025,11 +1040,11 @@
       <c r="E6" s="4">
         <v>313</v>
       </c>
-      <c r="F6" t="s">
+      <c r="J6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>56</v>
       </c>
@@ -1042,11 +1057,14 @@
       <c r="E7" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="J7" s="7" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>56</v>
       </c>
@@ -1059,11 +1077,11 @@
       <c r="E8" s="4">
         <v>34</v>
       </c>
-      <c r="F8" t="s">
+      <c r="J8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>56</v>
       </c>
@@ -1076,11 +1094,11 @@
       <c r="E9" s="4">
         <v>104</v>
       </c>
-      <c r="F9" t="s">
+      <c r="J9" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="C10" t="s">
         <v>59</v>
       </c>
@@ -1090,11 +1108,11 @@
       <c r="E10" s="4">
         <v>537</v>
       </c>
-      <c r="F10" t="s">
+      <c r="J10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>56</v>
       </c>
@@ -1107,11 +1125,11 @@
       <c r="E11" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="F11" t="s">
+      <c r="J11" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>56</v>
       </c>
@@ -1124,11 +1142,11 @@
       <c r="E12" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="F12" t="s">
+      <c r="J12" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>56</v>
       </c>
@@ -1141,11 +1159,11 @@
       <c r="E13" s="4">
         <v>532</v>
       </c>
-      <c r="F13" t="s">
+      <c r="J13" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>56</v>
       </c>
@@ -1158,11 +1176,11 @@
       <c r="E14" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="F14" t="s">
+      <c r="J14" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>56</v>
       </c>
@@ -1175,11 +1193,11 @@
       <c r="E15" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="F15" t="s">
+      <c r="J15" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>56</v>
       </c>
@@ -1192,11 +1210,11 @@
       <c r="E16" s="4">
         <v>220</v>
       </c>
-      <c r="F16" t="s">
+      <c r="J16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>56</v>
       </c>
@@ -1209,11 +1227,11 @@
       <c r="E17" s="4">
         <v>151</v>
       </c>
-      <c r="F17" t="s">
+      <c r="J17" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>56</v>
       </c>
@@ -1226,11 +1244,11 @@
       <c r="E18" s="4">
         <v>395</v>
       </c>
-      <c r="F18" t="s">
+      <c r="J18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>56</v>
       </c>
@@ -1243,11 +1261,11 @@
       <c r="E19" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F19" t="s">
+      <c r="J19" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>56</v>
       </c>
@@ -1260,11 +1278,11 @@
       <c r="E20" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="F20" t="s">
+      <c r="J20" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>56</v>
       </c>
@@ -1277,11 +1295,11 @@
       <c r="E21" s="4">
         <v>349</v>
       </c>
-      <c r="F21" t="s">
+      <c r="J21" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>56</v>
       </c>
@@ -1294,11 +1312,11 @@
       <c r="E22" s="4">
         <v>354</v>
       </c>
-      <c r="F22" t="s">
+      <c r="J22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>56</v>
       </c>
@@ -1311,11 +1329,11 @@
       <c r="E23" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="F23" t="s">
+      <c r="J23" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>56</v>
       </c>
@@ -1328,11 +1346,11 @@
       <c r="E24" s="4">
         <v>429</v>
       </c>
-      <c r="F24" t="s">
+      <c r="J24" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>56</v>
       </c>
@@ -1345,11 +1363,11 @@
       <c r="E25" s="4">
         <v>193</v>
       </c>
-      <c r="F25" t="s">
+      <c r="J25" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>56</v>
       </c>
@@ -1362,11 +1380,11 @@
       <c r="E26" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="F26" t="s">
+      <c r="J26" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>56</v>
       </c>
@@ -1379,11 +1397,11 @@
       <c r="E27" s="4">
         <v>256</v>
       </c>
-      <c r="F27" t="s">
+      <c r="J27" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>56</v>
       </c>
@@ -1396,11 +1414,11 @@
       <c r="E28" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="F28" t="s">
+      <c r="J28" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>56</v>
       </c>
@@ -1413,11 +1431,11 @@
       <c r="E29" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="F29" t="s">
+      <c r="J29" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>56</v>
       </c>
@@ -1430,11 +1448,11 @@
       <c r="E30" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="F30" t="s">
+      <c r="J30" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>56</v>
       </c>
@@ -1447,11 +1465,11 @@
       <c r="E31" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="F31" t="s">
+      <c r="J31" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>56</v>
       </c>
@@ -1464,11 +1482,11 @@
       <c r="E32" s="4">
         <v>475</v>
       </c>
-      <c r="F32" t="s">
+      <c r="J32" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>56</v>
       </c>
@@ -1481,11 +1499,11 @@
       <c r="E33" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="F33" t="s">
+      <c r="J33" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>56</v>
       </c>
@@ -1498,11 +1516,11 @@
       <c r="E34" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="F34" t="s">
+      <c r="J34" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>56</v>
       </c>
@@ -1518,11 +1536,11 @@
       <c r="E35" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="F35" t="s">
+      <c r="J35" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>56</v>
       </c>
@@ -1538,11 +1556,11 @@
       <c r="E36" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="F36" t="s">
+      <c r="J36" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>56</v>
       </c>
@@ -1555,11 +1573,11 @@
       <c r="E37" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="F37" t="s">
+      <c r="J37" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>56</v>
       </c>
@@ -1572,11 +1590,11 @@
       <c r="E38" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="F38" t="s">
+      <c r="J38" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>56</v>
       </c>
@@ -1589,11 +1607,11 @@
       <c r="E39" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="F39" t="s">
+      <c r="J39" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>56</v>
       </c>
@@ -1606,11 +1624,11 @@
       <c r="E40" s="4">
         <v>488</v>
       </c>
-      <c r="F40" t="s">
+      <c r="J40" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>56</v>
       </c>
@@ -1623,11 +1641,11 @@
       <c r="E41" s="4">
         <v>284</v>
       </c>
-      <c r="F41" t="s">
+      <c r="J41" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>56</v>
       </c>
@@ -1640,11 +1658,11 @@
       <c r="E42" s="4">
         <v>23</v>
       </c>
-      <c r="F42" t="s">
+      <c r="J42" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>56</v>
       </c>
@@ -1657,11 +1675,11 @@
       <c r="E43" s="4">
         <v>65</v>
       </c>
-      <c r="F43" t="s">
+      <c r="J43" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>56</v>
       </c>
@@ -1674,11 +1692,11 @@
       <c r="E44" s="4">
         <v>368</v>
       </c>
-      <c r="F44" t="s">
+      <c r="J44" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>56</v>
       </c>
@@ -1691,11 +1709,11 @@
       <c r="E45" s="4">
         <v>363</v>
       </c>
-      <c r="F45" t="s">
+      <c r="J45" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>56</v>
       </c>
@@ -1708,11 +1726,11 @@
       <c r="E46" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="F46" t="s">
+      <c r="J46" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>56</v>
       </c>
@@ -1725,11 +1743,11 @@
       <c r="E47" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="F47" t="s">
+      <c r="J47" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>56</v>
       </c>
@@ -1742,7 +1760,7 @@
       <c r="E48" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="F48" t="s">
+      <c r="J48" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1753,12 +1771,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53C8A44C-B798-4416-9AA8-07AAF9D050FB}">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.7265625" style="1" customWidth="1"/>
     <col min="2" max="2" width="8.7265625" style="5"/>
-    <col min="3" max="3" width="16.08984375" customWidth="1"/>
+    <col min="3" max="3" width="16.08984375" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -1794,7 +1812,7 @@
       <c r="B4" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="4" t="s">
         <v>135</v>
       </c>
       <c r="D4" t="s">
@@ -1808,7 +1826,7 @@
       <c r="B5" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="4" t="s">
         <v>135</v>
       </c>
       <c r="D5" t="s">
@@ -1822,7 +1840,7 @@
       <c r="B6" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="4" t="s">
         <v>150</v>
       </c>
       <c r="D6" t="s">
@@ -1836,7 +1854,7 @@
       <c r="B7" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="4" t="s">
         <v>151</v>
       </c>
       <c r="D7" t="s">
@@ -1850,7 +1868,7 @@
       <c r="B8" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="4" t="s">
         <v>152</v>
       </c>
       <c r="D8" t="s">
@@ -1875,7 +1893,7 @@
       <c r="A10" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="4" t="s">
         <v>141</v>
       </c>
       <c r="D10" t="s">
@@ -1886,7 +1904,7 @@
       <c r="A11" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="4" t="s">
         <v>85</v>
       </c>
       <c r="D11" s="6" t="s">
@@ -1900,7 +1918,7 @@
       <c r="A12" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="4" t="s">
         <v>142</v>
       </c>
       <c r="D12" t="s">
@@ -1914,7 +1932,7 @@
       <c r="A13" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="4" t="s">
         <v>145</v>
       </c>
       <c r="D13" t="s">
@@ -1928,7 +1946,7 @@
       <c r="A14" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="4" t="s">
         <v>142</v>
       </c>
       <c r="D14" t="s">
@@ -1942,7 +1960,7 @@
       <c r="A15" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="4" t="s">
         <v>159</v>
       </c>
       <c r="D15" t="s">
@@ -1950,6 +1968,20 @@
       </c>
       <c r="G15" t="s">
         <v>160</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C16" s="4">
+        <v>507</v>
+      </c>
+      <c r="D16" t="s">
+        <v>163</v>
+      </c>
+      <c r="G16" t="s">
+        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
annotations on phoenix cave playtesting
</commit_message>
<xml_diff>
--- a/claude_reference/Ruin_playtesting_checklist.xlsx
+++ b/claude_reference/Ruin_playtesting_checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hansr\Documents\GitHub\WorldsCollide\claude_reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0AA8BB6-3D80-451F-A22B-0249657EB27F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C260FEA-87A4-4D04-B244-1EC735544C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{690EC4E7-DE9A-4E52-B9DA-56D934A5EC63}"/>
+    <workbookView xWindow="3000" yWindow="3000" windowWidth="19200" windowHeight="11170" xr2:uid="{690EC4E7-DE9A-4E52-B9DA-56D934A5EC63}"/>
   </bookViews>
   <sheets>
     <sheet name="Rewards" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Update Narshe ruination rooms
Was missing moogle room & had Lone Wolf reward in the wrong room.
</commit_message>
<xml_diff>
--- a/claude_reference/Ruin_playtesting_checklist.xlsx
+++ b/claude_reference/Ruin_playtesting_checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hansr\Documents\GitHub\WorldsCollide\claude_reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B919E58-1CE6-4E62-92DD-1FFA57766E22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54341C4B-5422-43FE-8EC2-5C5B65CCED17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="19200" windowHeight="11170" xr2:uid="{690EC4E7-DE9A-4E52-B9DA-56D934A5EC63}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{690EC4E7-DE9A-4E52-B9DA-56D934A5EC63}"/>
   </bookViews>
   <sheets>
     <sheet name="Rewards" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
bugfix two rewards in room '41a'
It's ok, but the ROOM_REWARD dictionary needs to be defined correctly.  It had been overwriting the Lone Wolf entry with the Tritoch one.
</commit_message>
<xml_diff>
--- a/claude_reference/Ruin_playtesting_checklist.xlsx
+++ b/claude_reference/Ruin_playtesting_checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hansr\Documents\GitHub\WorldsCollide\claude_reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D40A1996-A4AC-4375-86C9-62C339F19EC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1EE6695-D68A-45CF-8174-C621E8ED8F2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{690EC4E7-DE9A-4E52-B9DA-56D934A5EC63}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="174">
   <si>
     <t>PLAYTESTING CHECKLIST: Rewards in -ruin mode</t>
   </si>
@@ -559,24 +559,6 @@
   </si>
   <si>
     <t>Had to turn off y-swap while inside</t>
-  </si>
-  <si>
-    <t>Works, but need to add invisible blocker or something on umaro cave exit to prevent leaving the screen.</t>
-  </si>
-  <si>
-    <t>Works, but need to add invisible blocker or something oo umaro cave exit to prevent leaving the screen.</t>
-  </si>
-  <si>
-    <t>Works, but need to add invisible blocker or something ma umaro cave exit to prevent leaving the screen.</t>
-  </si>
-  <si>
-    <t>Works, but need to add invisible blocker or something ri umaro cave exit to prevent leaving the screen.</t>
-  </si>
-  <si>
-    <t>Works, but need to add invisible blocker or something ze umaro cave exit to prevent leaving the screen.</t>
-  </si>
-  <si>
-    <t>Works, but need to add invisible blocker or something uc umaro cave exit to prevent leaving the screen.</t>
   </si>
 </sst>
 </file>
@@ -1834,7 +1816,7 @@
         <v>50</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>159</v>
+        <v>50</v>
       </c>
       <c r="C42" t="s">
         <v>112</v>
@@ -1845,9 +1827,7 @@
       <c r="E42" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="F42" s="10" t="s">
-        <v>174</v>
-      </c>
+      <c r="F42" s="10"/>
       <c r="J42" s="7" t="s">
         <v>172</v>
       </c>

</xml_diff>

<commit_message>
playtesting Lone Wolf complete
Bugfix complete for bridge blocker, cliff blocker, and y-switch.  Tested with esper & character route.
Also simplified code and fixed issue with overwriting wor_pair in maps.postprocess_door_maps().
</commit_message>
<xml_diff>
--- a/claude_reference/Ruin_playtesting_checklist.xlsx
+++ b/claude_reference/Ruin_playtesting_checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hansr\Documents\GitHub\WorldsCollide\claude_reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1EE6695-D68A-45CF-8174-C621E8ED8F2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAB0FE6E-441A-49B0-BC13-6EF11865DEB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{690EC4E7-DE9A-4E52-B9DA-56D934A5EC63}"/>
+    <workbookView xWindow="-26910" yWindow="1620" windowWidth="16305" windowHeight="15765" xr2:uid="{690EC4E7-DE9A-4E52-B9DA-56D934A5EC63}"/>
   </bookViews>
   <sheets>
     <sheet name="Rewards" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Ruination: character recruiting playtesting complete!
- haven't done an actual full run yet.
- Should still debug the "Remote character gating" issues.  We generally don't want that.
</commit_message>
<xml_diff>
--- a/claude_reference/Ruin_playtesting_checklist.xlsx
+++ b/claude_reference/Ruin_playtesting_checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hansr\Documents\GitHub\WorldsCollide\claude_reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAB0FE6E-441A-49B0-BC13-6EF11865DEB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94AF2A32-0F51-4960-BA79-8F08BFCA17FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26910" yWindow="1620" windowWidth="16305" windowHeight="15765" xr2:uid="{690EC4E7-DE9A-4E52-B9DA-56D934A5EC63}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{690EC4E7-DE9A-4E52-B9DA-56D934A5EC63}"/>
   </bookViews>
   <sheets>
     <sheet name="Rewards" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="174">
   <si>
     <t>PLAYTESTING CHECKLIST: Rewards in -ruin mode</t>
   </si>
@@ -1856,6 +1856,9 @@
       <c r="A44" s="1" t="s">
         <v>50</v>
       </c>
+      <c r="B44" s="3" t="s">
+        <v>50</v>
+      </c>
       <c r="C44" t="s">
         <v>115</v>
       </c>
@@ -1873,6 +1876,9 @@
       <c r="A45" s="1" t="s">
         <v>50</v>
       </c>
+      <c r="B45" s="3" t="s">
+        <v>50</v>
+      </c>
       <c r="C45" t="s">
         <v>117</v>
       </c>
@@ -1890,6 +1896,9 @@
       <c r="A46" s="1" t="s">
         <v>50</v>
       </c>
+      <c r="B46" s="3" t="s">
+        <v>50</v>
+      </c>
       <c r="C46" t="s">
         <v>119</v>
       </c>
@@ -1907,6 +1916,9 @@
       <c r="A47" s="1" t="s">
         <v>50</v>
       </c>
+      <c r="B47" s="3" t="s">
+        <v>50</v>
+      </c>
       <c r="C47" t="s">
         <v>119</v>
       </c>
@@ -1922,6 +1934,9 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B48" s="3" t="s">
         <v>50</v>
       </c>
       <c r="C48" t="s">

</xml_diff>

<commit_message>
Implementing local character gating A
Implemented local character gating for TERRA, LOCKE, EDGAR
- Lete River (does not attack without TERRA)
- TunnelArmr (does not attack without LOCKE)
- Engine Room (cannot enter without EDGAR)
- Ancient Castle (statue unresponsive without EDGAR)
</commit_message>
<xml_diff>
--- a/claude_reference/Ruin_playtesting_checklist.xlsx
+++ b/claude_reference/Ruin_playtesting_checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hansr\Documents\GitHub\WorldsCollide\claude_reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94AF2A32-0F51-4960-BA79-8F08BFCA17FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{532C5DD5-8AAF-44EA-A118-E8033FBCD1DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{690EC4E7-DE9A-4E52-B9DA-56D934A5EC63}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="18240" activeTab="1" xr2:uid="{690EC4E7-DE9A-4E52-B9DA-56D934A5EC63}"/>
   </bookViews>
   <sheets>
     <sheet name="Rewards" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="179">
   <si>
     <t>PLAYTESTING CHECKLIST: Rewards in -ruin mode</t>
   </si>
@@ -559,6 +559,21 @@
   </si>
   <si>
     <t>Had to turn off y-swap while inside</t>
+  </si>
+  <si>
+    <t>If LOCKE not recruited, TunnelArmr should not trigger.</t>
+  </si>
+  <si>
+    <t>LOCAL CHARACTER GATING UPDATES:</t>
+  </si>
+  <si>
+    <t>If TERRA not recruited, Ultros should not trigger.</t>
+  </si>
+  <si>
+    <t>If EDGAR not recruited, cannot enter the basement.</t>
+  </si>
+  <si>
+    <t>If EDGAR not recruited, statue does nothing.</t>
   </si>
 </sst>
 </file>
@@ -1959,7 +1974,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53C8A44C-B798-4416-9AA8-07AAF9D050FB}">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.7265625" style="1" customWidth="1"/>
@@ -2217,6 +2232,55 @@
         <v>170</v>
       </c>
     </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D22" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C23" s="4">
+        <v>104</v>
+      </c>
+      <c r="D23" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D24" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25" s="4">
+        <v>532</v>
+      </c>
+      <c r="D25" t="s">
+        <v>178</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>